<commit_message>
Ampliar catálogo de gráficos y añadir copia a PowerPoint como EMF
- Desplegable de tipo de gráfico ampliado a 7 tipos drop-in (Columnas, Barras,
  Líneas, Área, Circular, Anillo, Radar).
- Macro: mapeo completo de tipos, cambio sin parpadeo (ScreenUpdating) y nueva
  CopiarAPowerPoint que pega el gráfico como EMF vectorial (sin vínculos, no se
  rompe) vía late binding.
- catalogo_graficos.md: qué gráficos usar en una gestora (incl. multi-serie para
  Fase 2: apiladas, combo, dispersión riesgo/retorno, waterfall), razonamiento
  EMF y notas de UX/rendimiento.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01343tRzXDqve9dfZ8CoRemv
</commit_message>
<xml_diff>
--- a/bq-excel-charts/excel-nativo/Panel_Interactivo.xlsx
+++ b/bq-excel-charts/excel-nativo/Panel_Interactivo.xlsx
@@ -624,7 +624,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Verticales</t>
+          <t>Columnas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -686,7 +686,7 @@
       <formula1>=INDIRECT($B$3)</formula1>
     </dataValidation>
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Verticales,Horizontales"</formula1>
+      <formula1>"Columnas,Barras,Líneas,Área,Circular,Anillo,Radar"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>